<commit_message>
feat: unified legal claim engine, cancelled contract reactivation, traffic violations-only claim scope, and legal transfer readiness hardening
</commit_message>
<xml_diff>
--- a/معتمدون-ملفات-موقعة.xlsx
+++ b/معتمدون-ملفات-موقعة.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet name="ملخص الملفات" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="المعتمدون" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="عقود سابقة على نفس المركبة" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ملخص" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="عقود نشطة" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="قرارات خميس" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="عقود سابقة على نفس المركبة" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ملخص" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="عقود نشطة" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'المعتمدون'!$A$1:$Z$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'المعتمدون'!$A$1:$AB$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'المعتمدون'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'عقود سابقة على نفس المركبة'!$A$1:$O$91</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'عقود سابقة على نفس المركبة'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'عقود نشطة'!$A$1:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'قرارات خميس'!$A$4:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'عقود سابقة على نفس المركبة'!$A$1:$O$91</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'عقود سابقة على نفس المركبة'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'عقود نشطة'!$A$1:$J$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,8 +102,48 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007B5800"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A365D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007B241C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001A365D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007B241C"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -183,6 +225,31 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7FBFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -238,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -371,6 +438,54 @@
     <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,6 +560,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>KHAMIS</author>
+  </authors>
+  <commentList>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>قرارات خميس للتقرير فقط. النظام الحي (Fleetify / قاعدة البيانات) لم يُعدَّل. أُلغي التنفيذ الحي بناءً على إلغاء خميس.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -736,7 +866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -759,7 +889,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -908,14 +1037,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -930,24 +1051,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
@@ -1039,11 +1142,93 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="46" t="inlineStr">
+        <is>
+          <t>قرارات خميس للتقرير — النظام الحي لم يُعدَّل</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="47" t="inlineStr">
+        <is>
+          <t>تاريخ التسجيل (توقيت الرياض)</t>
+        </is>
+      </c>
+      <c r="B52" s="47" t="inlineStr">
+        <is>
+          <t>2026-08-31 20:02</t>
+        </is>
+      </c>
+      <c r="C52" s="47" t="n"/>
+      <c r="D52" s="47" t="inlineStr">
+        <is>
+          <t>أُلغي التنفيذ الحي بناءً على إلغاء خميس. لا كتابة على Fleetify/Supabase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="47" t="inlineStr">
+        <is>
+          <t>عدد تعليمات خميس</t>
+        </is>
+      </c>
+      <c r="B53" s="47" t="n">
+        <v>28</v>
+      </c>
+      <c r="C53" s="47" t="n"/>
+      <c r="D53" s="47" t="inlineStr">
+        <is>
+          <t>كل التعليمات في ورقة «قرارات خميس»</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="47" t="inlineStr">
+        <is>
+          <t>تعليمات لها صف في المعتمدون</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C54" s="47" t="n"/>
+      <c r="D54" s="47" t="inlineStr">
+        <is>
+          <t>صفوف المعتمدون التي أُضيف إليها قرار: 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="47" t="inlineStr">
+        <is>
+          <t>تعليمات بلا صف في المعتمدون</t>
+        </is>
+      </c>
+      <c r="B55" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="47" t="n"/>
+      <c r="D55" s="47" t="inlineStr">
+        <is>
+          <t>أُضيفت في قرارات خميس فقط: C-ALF-0061؛ LTO2024103</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="49" t="inlineStr">
+        <is>
+          <t>أُضيف العمودان «قرار خميس» و«إجراء مطلوب» في ورقة المعتمدون (AA–AB) دون حذف تواريخ الورد أو عقد نشط أو مطابقة PDF. النص مسبوق بـ: قرار للتقرير — النظام الحي لم يُعدَّل.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A56:D56"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A51:D51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1055,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z79"/>
+  <dimension ref="A1:AB79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1081,6 +1266,8 @@
     <col width="24" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="78" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1214,8 +1401,18 @@
           <t>حالة العقد النشط</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>قرار خميس</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>إجراء مطلوب</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2782</t>
@@ -1318,8 +1515,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+      <c r="AA2" s="50" t="inlineStr">
+        <is>
+          <t>[7] قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء AGR-202504-399591. تحويل/إنشاء عقد جديد باسم سعيد الهلالي. (لوحة 2782 / شرفي عبد الله هو صاحب العقد الحي الحالي في «عقود سابقة»)</t>
+        </is>
+      </c>
+      <c r="AB2" s="51" t="inlineStr">
+        <is>
+          <t>[7] إلغاء AGR-202504-399591 + عقد جديد باسم سعيد الهلالي</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>603353</t>
@@ -1422,8 +1629,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+      <c r="AA3" s="50" t="inlineStr">
+        <is>
+          <t>[17] قرار للتقرير — النظام الحي لم يُعدَّل. العقد صحيح. اللوحة تغيّرت إلى عادية 603353.</t>
+        </is>
+      </c>
+      <c r="AB3" s="51" t="inlineStr">
+        <is>
+          <t>[17] اعتماد العقد + تحديث اللوحة إلى 603353</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>7066</t>
@@ -1528,6 +1745,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA4" s="50" t="inlineStr">
+        <is>
+          <t>[26] قرار للتقرير — النظام الحي لم يُعدَّل. تم دفع جميع المستحقات (حسب قرار خميس). تحويل المركبة باسمه.</t>
+        </is>
+      </c>
+      <c r="AB4" s="51" t="inlineStr">
+        <is>
+          <t>[26] تحويل المركبة باسمه (المستحقات مسددة حسب القرار)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1628,8 +1855,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
+      <c r="AA5" s="52" t="n"/>
+      <c r="AB5" s="52" t="n"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>862165</t>
@@ -1732,8 +1961,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
+      <c r="AA6" s="50" t="inlineStr">
+        <is>
+          <t>[19] قرار للتقرير — النظام الحي لم يُعدَّل. تعديل اسم العميل إلى مهدي الشريف عبد الرحيم يوسف.</t>
+        </is>
+      </c>
+      <c r="AB6" s="51" t="inlineStr">
+        <is>
+          <t>[19] تعديل اسم العميل</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>893409</t>
@@ -1844,8 +2083,18 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
+      <c r="AA7" s="50" t="inlineStr">
+        <is>
+          <t>[6] قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء العقد. إنشاء عقد جديد لنفس العميل. تاريخ البداية: ينتظر خميس.</t>
+        </is>
+      </c>
+      <c r="AB7" s="51" t="inlineStr">
+        <is>
+          <t>[6] إلغاء C-ALF-0030 + إنشاء عقد جديد (تاريخ البداية: ينتظر خميس)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>21860</t>
@@ -1964,8 +2213,18 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
+      <c r="AA8" s="50" t="inlineStr">
+        <is>
+          <t>[1] قرار للتقرير — النظام الحي لم يُعدَّل. العقد ملغي. تحويله للشؤون القانونية، وهنا فقط تُسجَّل المخالفات المرورية. إنشاء عقد جديد وتحويل الجديد للشؤون. تحويل المدفوعات على العقد الجديد. (كان نشط على 725473 في المطابقة السابقة)</t>
+        </is>
+      </c>
+      <c r="AB8" s="51" t="inlineStr">
+        <is>
+          <t>[1] إلغاء C-ALF-0069 + إنشاء عقد جديد + تحويل للشؤون + نقل المدفوعات والمخالفات</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>5890</t>
@@ -2070,6 +2329,16 @@
       <c r="Z9" s="41" t="inlineStr">
         <is>
           <t>لا يوجد عقد ساري</t>
+        </is>
+      </c>
+      <c r="AA9" s="50" t="inlineStr">
+        <is>
+          <t>[9] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل LTO2024340 إلى نشط. إلغاء LTO202410.</t>
+        </is>
+      </c>
+      <c r="AB9" s="51" t="inlineStr">
+        <is>
+          <t>[9] تحويل LTO2024340 إلى نشط + إلغاء LTO202410</t>
         </is>
       </c>
     </row>
@@ -2182,6 +2451,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA10" s="52" t="n"/>
+      <c r="AB10" s="52" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -2302,6 +2573,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA11" s="52" t="n"/>
+      <c r="AB11" s="52" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -2424,6 +2697,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA12" s="52" t="n"/>
+      <c r="AB12" s="52" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -2510,6 +2785,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA13" s="52" t="n"/>
+      <c r="AB13" s="52" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -2596,6 +2873,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA14" s="52" t="n"/>
+      <c r="AB14" s="52" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -2690,8 +2969,10 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+      <c r="AA15" s="52" t="n"/>
+      <c r="AB15" s="52" t="n"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>8204</t>
@@ -2776,8 +3057,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+      <c r="AA16" s="50" t="inlineStr">
+        <is>
+          <t>[22] قرار للتقرير — النظام الحي لم يُعدَّل. فتح بلاغ مستعجل.</t>
+        </is>
+      </c>
+      <c r="AB16" s="51" t="inlineStr">
+        <is>
+          <t>[22] فتح بلاغ مستعجل</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>846485</t>
@@ -2858,6 +3149,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA17" s="50" t="inlineStr">
+        <is>
+          <t>[27] قرار للتقرير — النظام الحي لم يُعدَّل. حذف هذا العقد.</t>
+        </is>
+      </c>
+      <c r="AB17" s="51" t="inlineStr">
+        <is>
+          <t>[27] حذف العقد</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -2940,6 +3241,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA18" s="52" t="n"/>
+      <c r="AB18" s="52" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -3024,8 +3327,10 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
+      <c r="AA19" s="52" t="n"/>
+      <c r="AB19" s="52" t="n"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>857051</t>
@@ -3110,6 +3415,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA20" s="50" t="inlineStr">
+        <is>
+          <t>[4] قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء العقد. يكون باسم فخري الدين عثمان.</t>
+        </is>
+      </c>
+      <c r="AB20" s="51" t="inlineStr">
+        <is>
+          <t>[4] إلغاء LTO2024152 + العقد باسم فخري الدين عثمان</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -3222,8 +3537,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
+      <c r="AA21" s="52" t="n"/>
+      <c r="AB21" s="52" t="n"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>5889</t>
@@ -3314,6 +3631,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA22" s="50" t="inlineStr">
+        <is>
+          <t>[8] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="AB22" s="51" t="inlineStr">
+        <is>
+          <t>[8] تحويل إلى نشط</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -3400,6 +3727,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA23" s="52" t="n"/>
+      <c r="AB23" s="52" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -3512,6 +3841,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA24" s="52" t="n"/>
+      <c r="AB24" s="52" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -3596,8 +3927,10 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
+      <c r="AA25" s="52" t="n"/>
+      <c r="AB25" s="52" t="n"/>
+    </row>
+    <row r="26" ht="48" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>11473</t>
@@ -3688,8 +4021,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
+      <c r="AA26" s="50" t="inlineStr">
+        <is>
+          <t>[18] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="AB26" s="51" t="inlineStr">
+        <is>
+          <t>[18] تحويل إلى نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>676281</t>
@@ -3792,8 +4135,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
+      <c r="AA27" s="50" t="inlineStr">
+        <is>
+          <t>[2] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد للشؤون القانونية.</t>
+        </is>
+      </c>
+      <c r="AB27" s="51" t="inlineStr">
+        <is>
+          <t>[2] تحويل للشؤون القانونية</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>7038</t>
@@ -3892,6 +4245,16 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA28" s="50" t="inlineStr">
+        <is>
+          <t>[11] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى مهدي محمد القاطري.</t>
+        </is>
+      </c>
+      <c r="AB28" s="51" t="inlineStr">
+        <is>
+          <t>[11] تحويل المركبة إلى مهدي محمد القاطري</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -3986,8 +4349,10 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
+      <c r="AA29" s="52" t="n"/>
+      <c r="AB29" s="52" t="n"/>
+    </row>
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>7058</t>
@@ -4090,8 +4455,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
+      <c r="AA30" s="50" t="inlineStr">
+        <is>
+          <t>[13] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="AB30" s="51" t="inlineStr">
+        <is>
+          <t>[13] تحويل إلى نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>7063</t>
@@ -4194,8 +4569,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
+      <c r="AA31" s="50" t="inlineStr">
+        <is>
+          <t>[14] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="AB31" s="51" t="inlineStr">
+        <is>
+          <t>[14] تحويل إلى نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>7071</t>
@@ -4284,8 +4669,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
+      <c r="AA32" s="50" t="inlineStr">
+        <is>
+          <t>[16] قرار للتقرير — النظام الحي لم يُعدَّل. مستعجل: كنسل المركبة + إجراء قانوني.</t>
+        </is>
+      </c>
+      <c r="AB32" s="51" t="inlineStr">
+        <is>
+          <t>[16] كنسل المركبة + إجراء قانوني (مستعجل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>847099</t>
@@ -4388,8 +4783,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
+      <c r="AA33" s="50" t="inlineStr">
+        <is>
+          <t>[21] قرار للتقرير — النظام الحي لم يُعدَّل. فتح بلاغ + كنسل المركبة.</t>
+        </is>
+      </c>
+      <c r="AB33" s="51" t="inlineStr">
+        <is>
+          <t>[21] فتح بلاغ + كنسل المركبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>893406</t>
@@ -4480,6 +4885,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA34" s="50" t="inlineStr">
+        <is>
+          <t>[5] قرار للتقرير — النظام الحي لم يُعدَّل. لوحة مفقودة. تم إبعاد محمود جاسم الصالح والمركبة لم تُرجع، عيال عمه ينكرون المكان.</t>
+        </is>
+      </c>
+      <c r="AB34" s="51" t="inlineStr">
+        <is>
+          <t>[5] تسجيل مركبة مفقودة + متابعة قانونية</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -4584,6 +4999,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA35" s="52" t="n"/>
+      <c r="AB35" s="52" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -4688,6 +5105,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA36" s="52" t="n"/>
+      <c r="AB36" s="52" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -4794,6 +5213,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA37" s="52" t="n"/>
+      <c r="AB37" s="52" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -4890,8 +5311,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
+      <c r="AA38" s="52" t="n"/>
+      <c r="AB38" s="52" t="n"/>
+    </row>
+    <row r="39" ht="48" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>185513</t>
@@ -5004,8 +5427,18 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
+      <c r="AA39" s="50" t="inlineStr">
+        <is>
+          <t>[25] قرار للتقرير — النظام الحي لم يُعدَّل. مخالفات مرورية. فتح قضية.</t>
+        </is>
+      </c>
+      <c r="AB39" s="51" t="inlineStr">
+        <is>
+          <t>[25] فتح قضية مخالفات مرورية</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>185573</t>
@@ -5108,6 +5541,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA40" s="50" t="inlineStr">
+        <is>
+          <t>[26] قرار للتقرير — النظام الحي لم يُعدَّل. تم دفع جميع المستحقات (حسب قرار خميس). تحويل المركبة باسمه.</t>
+        </is>
+      </c>
+      <c r="AB40" s="51" t="inlineStr">
+        <is>
+          <t>[26] تحويل المركبة باسمه (المستحقات مسددة حسب القرار)</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -5216,6 +5659,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA41" s="52" t="n"/>
+      <c r="AB41" s="52" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -5328,6 +5773,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA42" s="52" t="n"/>
+      <c r="AB42" s="52" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -5432,6 +5879,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA43" s="52" t="n"/>
+      <c r="AB43" s="52" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -5546,6 +5995,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA44" s="52" t="n"/>
+      <c r="AB44" s="52" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -5658,6 +6109,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA45" s="52" t="n"/>
+      <c r="AB45" s="52" t="n"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -5758,6 +6211,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA46" s="52" t="n"/>
+      <c r="AB46" s="52" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -5864,6 +6319,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA47" s="52" t="n"/>
+      <c r="AB47" s="52" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -5968,6 +6425,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA48" s="52" t="n"/>
+      <c r="AB48" s="52" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -6068,6 +6527,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA49" s="52" t="n"/>
+      <c r="AB49" s="52" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -6168,6 +6629,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA50" s="52" t="n"/>
+      <c r="AB50" s="52" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -6272,6 +6735,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA51" s="52" t="n"/>
+      <c r="AB51" s="52" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -6376,6 +6841,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA52" s="52" t="n"/>
+      <c r="AB52" s="52" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -6488,8 +6955,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="54" ht="22" customHeight="1">
+      <c r="AA53" s="52" t="n"/>
+      <c r="AB53" s="52" t="n"/>
+    </row>
+    <row r="54" ht="48" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>5900</t>
@@ -6580,6 +7049,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA54" s="50" t="inlineStr">
+        <is>
+          <t>[10] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى محمد عزيز محسن جلالي.</t>
+        </is>
+      </c>
+      <c r="AB54" s="51" t="inlineStr">
+        <is>
+          <t>[10] تحويل المركبة إلى محمد عزيز محسن جلالي</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -6682,6 +7161,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA55" s="52" t="n"/>
+      <c r="AB55" s="52" t="n"/>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -6782,6 +7263,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA56" s="52" t="n"/>
+      <c r="AB56" s="52" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -6894,6 +7377,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA57" s="52" t="n"/>
+      <c r="AB57" s="52" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -7006,8 +7491,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="59" ht="22" customHeight="1">
+      <c r="AA58" s="52" t="n"/>
+      <c r="AB58" s="52" t="n"/>
+    </row>
+    <row r="59" ht="48" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>7041</t>
@@ -7118,8 +7605,18 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="60" ht="22" customHeight="1">
+      <c r="AA59" s="50" t="inlineStr">
+        <is>
+          <t>[12] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى رمزي الهاشمي بعزاوي.</t>
+        </is>
+      </c>
+      <c r="AB59" s="51" t="inlineStr">
+        <is>
+          <t>[12] تحويل المركبة إلى رمزي الهاشمي بعزاوي</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="48" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>7043</t>
@@ -7228,6 +7725,16 @@
       <c r="Z60" s="42" t="inlineStr">
         <is>
           <t>ساري</t>
+        </is>
+      </c>
+      <c r="AA60" s="50" t="inlineStr">
+        <is>
+          <t>[23] قرار للتقرير — النظام الحي لم يُعدَّل. تعديل الاسم في النظام: حمد البشير يانس → حمزة البشير يانس.</t>
+        </is>
+      </c>
+      <c r="AB60" s="51" t="inlineStr">
+        <is>
+          <t>[23] تعديل الاسم: حمد → حمزة البشير يانس</t>
         </is>
       </c>
     </row>
@@ -7322,6 +7829,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA61" s="52" t="n"/>
+      <c r="AB61" s="52" t="n"/>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -7434,6 +7943,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA62" s="52" t="n"/>
+      <c r="AB62" s="52" t="n"/>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -7546,8 +8057,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="64" ht="22" customHeight="1">
+      <c r="AA63" s="52" t="n"/>
+      <c r="AB63" s="52" t="n"/>
+    </row>
+    <row r="64" ht="48" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>7060</t>
@@ -7638,8 +8151,18 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
-    </row>
-    <row r="65" ht="22" customHeight="1">
+      <c r="AA64" s="50" t="inlineStr">
+        <is>
+          <t>[24] قرار للتقرير — النظام الحي لم يُعدَّل. سيارة مفقودة.</t>
+        </is>
+      </c>
+      <c r="AB64" s="51" t="inlineStr">
+        <is>
+          <t>[24] تسجيل سيارة مفقودة</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="48" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
           <t>706150</t>
@@ -7730,6 +8253,16 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA65" s="50" t="inlineStr">
+        <is>
+          <t>[3] قرار للتقرير — النظام الحي لم يُعدَّل. C-ALF-0058 ملغي، لا مطالبات. المخالفات المرورية تُحوَّل إلى ألياس يعقوبي. HIST-XLS-ELIAS-706150 (في الملف: HIST-XLS-B70-706150) يُحوَّل إلى نشط وتُنقل عليه مخالفات 2026؛ القديم على العميل المعني. البحث عن المخالفات لتحويلها على العقد الصحيح.</t>
+        </is>
+      </c>
+      <c r="AB65" s="51" t="inlineStr">
+        <is>
+          <t>[3] إلغاء C-ALF-0058 (لا مطالبات) + تفعيل عقد ألياس + نقل مخالفات 2026 + جرد المخالفات</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -7842,6 +8375,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA66" s="52" t="n"/>
+      <c r="AB66" s="52" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -7946,6 +8481,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA67" s="52" t="n"/>
+      <c r="AB67" s="52" t="n"/>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -8058,6 +8595,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA68" s="52" t="n"/>
+      <c r="AB68" s="52" t="n"/>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
@@ -8170,6 +8709,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA69" s="52" t="n"/>
+      <c r="AB69" s="52" t="n"/>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -8276,6 +8817,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA70" s="52" t="n"/>
+      <c r="AB70" s="52" t="n"/>
     </row>
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -8388,8 +8931,10 @@
           <t>ساري</t>
         </is>
       </c>
-    </row>
-    <row r="72" ht="22" customHeight="1">
+      <c r="AA71" s="52" t="n"/>
+      <c r="AB71" s="52" t="n"/>
+    </row>
+    <row r="72" ht="48" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>8207</t>
@@ -8498,6 +9043,16 @@
       <c r="Z72" s="42" t="inlineStr">
         <is>
           <t>ساري</t>
+        </is>
+      </c>
+      <c r="AA72" s="50" t="inlineStr">
+        <is>
+          <t>[28] قرار للتقرير — النظام الحي لم يُعدَّل. تحويل للشؤون القانونية. المركبة للعميل. تعديل المتأخرات فقط: 5 أشهر. سُدد 2000 من المتأخرات. المركبة بيعت → خارج الخدمة.</t>
+        </is>
+      </c>
+      <c r="AB72" s="51" t="inlineStr">
+        <is>
+          <t>[28] تحويل للشؤون + متأخرات 5 أشهر (سُدد 2000) + المركبة خارج الخدمة</t>
         </is>
       </c>
     </row>
@@ -8600,6 +9155,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA73" s="52" t="n"/>
+      <c r="AB73" s="52" t="n"/>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -8712,6 +9269,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA74" s="52" t="n"/>
+      <c r="AB74" s="52" t="n"/>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
@@ -8824,6 +9383,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA75" s="52" t="n"/>
+      <c r="AB75" s="52" t="n"/>
     </row>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -8932,6 +9493,8 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA76" s="52" t="n"/>
+      <c r="AB76" s="52" t="n"/>
     </row>
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -9024,6 +9587,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA77" s="52" t="n"/>
+      <c r="AB77" s="52" t="n"/>
     </row>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
@@ -9120,6 +9685,8 @@
           <t>لا يوجد عقد ساري</t>
         </is>
       </c>
+      <c r="AA78" s="52" t="n"/>
+      <c r="AB78" s="52" t="n"/>
     </row>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
@@ -9220,15 +9787,1274 @@
           <t>ساري</t>
         </is>
       </c>
+      <c r="AA79" s="52" t="n"/>
+      <c r="AB79" s="52" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z79"/>
+  <autoFilter ref="A1:AB79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C0392B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="53" t="inlineStr">
+        <is>
+          <t>قرارات خميس للتقرير — النظام الحي لم يُعدَّل (Fleetify / العقود / المدفوعات / المخالفات لم تُمسّ). أُلغي التنفيذ الحي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="54" t="inlineStr">
+        <is>
+          <t>تسجيل 2026-08-31 20:02 (توقيت الرياض). هذه خطة عمل للتقرير فقط وليست حالة منفَّذة في النظام. المطابقة من أعمدة المعتمدون الحالية (الاسم / اللوحة / رقم العقد / عقد حي على لوحة أخرى) ومن ورقة «عقود سابقة على نفس المركبة» عند الحاجة. لم يُحذف أي عمود قائم (تواريخ الورد، عقد نشط، مطابقة PDF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>اسم</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>لوحة</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>رقم العقد</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>القرار (للتقرير — النظام الحي لم يُعدَّل)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>إجراء مطلوب</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>مطابقة المعتمدون</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>ملاحظة المطابقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>محمد ضياء العويني</t>
+        </is>
+      </c>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>725473 / 21860</t>
+        </is>
+      </c>
+      <c r="D5" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0069</t>
+        </is>
+      </c>
+      <c r="E5" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. العقد ملغي. تحويله للشؤون القانونية، وهنا فقط تُسجَّل المخالفات المرورية. إنشاء عقد جديد وتحويل الجديد للشؤون. تحويل المدفوعات على العقد الجديد. (كان نشط على 725473 في المطابقة السابقة)</t>
+        </is>
+      </c>
+      <c r="F5" s="56" t="inlineStr">
+        <is>
+          <t>إلغاء C-ALF-0069 + إنشاء عقد جديد + تحويل للشؤون + نقل المدفوعات والمخالفات</t>
+        </is>
+      </c>
+      <c r="G5" s="56" t="inlineStr">
+        <is>
+          <t>صف 8؛ محمد ضياء العويني؛ لوحة 21860؛ عقد AGR-202502-0426</t>
+        </is>
+      </c>
+      <c r="H5" s="56" t="inlineStr">
+        <is>
+          <t>مطابقة: صف المعتمدون بالاسم / C-ALF-0069 / 725473</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="57" t="inlineStr">
+        <is>
+          <t>حمزة بادو</t>
+        </is>
+      </c>
+      <c r="C6" s="57" t="inlineStr">
+        <is>
+          <t>676281</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="inlineStr">
+        <is>
+          <t>LTO202437</t>
+        </is>
+      </c>
+      <c r="E6" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد للشؤون القانونية.</t>
+        </is>
+      </c>
+      <c r="F6" s="57" t="inlineStr">
+        <is>
+          <t>تحويل للشؤون القانونية</t>
+        </is>
+      </c>
+      <c r="G6" s="57" t="inlineStr">
+        <is>
+          <t>صف 27؛ حمزة بادو؛ لوحة 676281؛ عقد LTO202437</t>
+        </is>
+      </c>
+      <c r="H6" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1">
+      <c r="A7" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>ألياس يعقوبي / مروان باكير (C-ALF-0058)</t>
+        </is>
+      </c>
+      <c r="C7" s="56" t="inlineStr">
+        <is>
+          <t>706150</t>
+        </is>
+      </c>
+      <c r="D7" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0058 + HIST-XLS-B70-706150 (المذكور HIST-XLS-ELIAS-706150)</t>
+        </is>
+      </c>
+      <c r="E7" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. C-ALF-0058 ملغي، لا مطالبات. المخالفات المرورية تُحوَّل إلى ألياس يعقوبي. HIST-XLS-ELIAS-706150 (في الملف: HIST-XLS-B70-706150) يُحوَّل إلى نشط وتُنقل عليه مخالفات 2026؛ القديم على العميل المعني. البحث عن المخالفات لتحويلها على العقد الصحيح.</t>
+        </is>
+      </c>
+      <c r="F7" s="56" t="inlineStr">
+        <is>
+          <t>إلغاء C-ALF-0058 (لا مطالبات) + تفعيل عقد ألياس + نقل مخالفات 2026 + جرد المخالفات</t>
+        </is>
+      </c>
+      <c r="G7" s="56" t="inlineStr">
+        <is>
+          <t>صف 65؛ ألياس يعقوبي؛ لوحة 706150؛ عقد HIST-XLS-B70-706150</t>
+        </is>
+      </c>
+      <c r="H7" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0058 موجود في «عقود سابقة» على نفس اللوحة باسم مروان باكير — ليس صفاً مستقلاً في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="57" t="inlineStr">
+        <is>
+          <t>فخري الدين عثمان (حالياً هاني هشام على LTO2024152)</t>
+        </is>
+      </c>
+      <c r="C8" s="57" t="inlineStr">
+        <is>
+          <t>857051</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024152</t>
+        </is>
+      </c>
+      <c r="E8" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء العقد. يكون باسم فخري الدين عثمان.</t>
+        </is>
+      </c>
+      <c r="F8" s="57" t="inlineStr">
+        <is>
+          <t>إلغاء LTO2024152 + العقد باسم فخري الدين عثمان</t>
+        </is>
+      </c>
+      <c r="G8" s="57" t="inlineStr">
+        <is>
+          <t>صف 20؛ فخري الدين عثمان؛ لوحة 857051؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H8" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024152 في «عقود سابقة» على اللوحة 857051 باسم هاني هشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1">
+      <c r="A9" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t>محمود جاسم الصالح</t>
+        </is>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>893406</t>
+        </is>
+      </c>
+      <c r="D9" s="56" t="inlineStr">
+        <is>
+          <t>HIST-XLS-B70-893406</t>
+        </is>
+      </c>
+      <c r="E9" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. لوحة مفقودة. تم إبعاد محمود جاسم الصالح والمركبة لم تُرجع، عيال عمه ينكرون المكان.</t>
+        </is>
+      </c>
+      <c r="F9" s="56" t="inlineStr">
+        <is>
+          <t>تسجيل مركبة مفقودة + متابعة قانونية</t>
+        </is>
+      </c>
+      <c r="G9" s="56" t="inlineStr">
+        <is>
+          <t>صف 34؛ محمود جاسم الصالح؛ لوحة 893406؛ عقد HIST-XLS-B70-893406</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="57" t="inlineStr">
+        <is>
+          <t>عقبة يوسف قصعاوي</t>
+        </is>
+      </c>
+      <c r="C10" s="57" t="inlineStr">
+        <is>
+          <t>893409 / 381247</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>C-ALF-0030</t>
+        </is>
+      </c>
+      <c r="E10" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء العقد. إنشاء عقد جديد لنفس العميل. تاريخ البداية: ينتظر خميس.</t>
+        </is>
+      </c>
+      <c r="F10" s="57" t="inlineStr">
+        <is>
+          <t>إلغاء C-ALF-0030 + إنشاء عقد جديد (تاريخ البداية: ينتظر خميس)</t>
+        </is>
+      </c>
+      <c r="G10" s="57" t="inlineStr">
+        <is>
+          <t>صف 7؛ عقبة يوسف قصعاوي؛ لوحة 893409؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H10" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
+      <c r="A11" s="55" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>سعيد الهلالي (العقد الحي الحالي: شرفي عبد الله)</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>2782</t>
+        </is>
+      </c>
+      <c r="D11" s="56" t="inlineStr">
+        <is>
+          <t>AGR-202504-399591</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء AGR-202504-399591. تحويل/إنشاء عقد جديد باسم سعيد الهلالي. (لوحة 2782 / شرفي عبد الله هو صاحب العقد الحي الحالي في «عقود سابقة»)</t>
+        </is>
+      </c>
+      <c r="F11" s="56" t="inlineStr">
+        <is>
+          <t>إلغاء AGR-202504-399591 + عقد جديد باسم سعيد الهلالي</t>
+        </is>
+      </c>
+      <c r="G11" s="56" t="inlineStr">
+        <is>
+          <t>صف 2؛ سعيد الهلالي؛ لوحة 2782؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="inlineStr">
+        <is>
+          <t>AGR-202504-399591 في «عقود سابقة» على 2782 باسم شرفي عبد الله — ليس رقم عقد في صف المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
+      <c r="A12" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="57" t="inlineStr">
+        <is>
+          <t>ايمن خليفة حمادي</t>
+        </is>
+      </c>
+      <c r="C12" s="57" t="inlineStr">
+        <is>
+          <t>5889</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="inlineStr">
+        <is>
+          <t>LTO202427</t>
+        </is>
+      </c>
+      <c r="E12" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="F12" s="57" t="inlineStr">
+        <is>
+          <t>تحويل إلى نشط</t>
+        </is>
+      </c>
+      <c r="G12" s="57" t="inlineStr">
+        <is>
+          <t>صف 22؛ ايمن خليفة حمادي؛ لوحة 5889؛ عقد LTO202427</t>
+        </is>
+      </c>
+      <c r="H12" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
+      <c r="A13" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>عبد العزيز بن نبيل جرفال</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>5890 / 17216</t>
+        </is>
+      </c>
+      <c r="D13" s="56" t="inlineStr">
+        <is>
+          <t>LTO2024340 + إلغاء LTO202410</t>
+        </is>
+      </c>
+      <c r="E13" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل LTO2024340 إلى نشط. إلغاء LTO202410.</t>
+        </is>
+      </c>
+      <c r="F13" s="56" t="inlineStr">
+        <is>
+          <t>تحويل LTO2024340 إلى نشط + إلغاء LTO202410</t>
+        </is>
+      </c>
+      <c r="G13" s="56" t="inlineStr">
+        <is>
+          <t>صف 9؛ عبد العزيز بن نبيل جرفال؛ لوحة 5890؛ عقد LTO2024340</t>
+        </is>
+      </c>
+      <c r="H13" s="56" t="inlineStr">
+        <is>
+          <t>LTO202410 ظاهر كعقد حي على لوحة أخرى (17216) في صف 5890</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
+      <c r="A14" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="57" t="inlineStr">
+        <is>
+          <t>محمد عزيز محسن جلالي</t>
+        </is>
+      </c>
+      <c r="C14" s="57" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
+      <c r="D14" s="57" t="inlineStr">
+        <is>
+          <t>HIST-XLS-T77-5900</t>
+        </is>
+      </c>
+      <c r="E14" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى محمد عزيز محسن جلالي.</t>
+        </is>
+      </c>
+      <c r="F14" s="57" t="inlineStr">
+        <is>
+          <t>تحويل المركبة إلى محمد عزيز محسن جلالي</t>
+        </is>
+      </c>
+      <c r="G14" s="57" t="inlineStr">
+        <is>
+          <t>صف 54؛ محمد عزيز محسن جلالي؛ لوحة 5900؛ عقد HIST-XLS-T77-5900</t>
+        </is>
+      </c>
+      <c r="H14" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="56" customHeight="1">
+      <c r="A15" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t>مهدي محمد القاطري (العقد الحي الحالي: ثامر محمد السيد / C-ALF-0048)</t>
+        </is>
+      </c>
+      <c r="C15" s="56" t="inlineStr">
+        <is>
+          <t>7038</t>
+        </is>
+      </c>
+      <c r="D15" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0048</t>
+        </is>
+      </c>
+      <c r="E15" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى مهدي محمد القاطري.</t>
+        </is>
+      </c>
+      <c r="F15" s="56" t="inlineStr">
+        <is>
+          <t>تحويل المركبة إلى مهدي محمد القاطري</t>
+        </is>
+      </c>
+      <c r="G15" s="56" t="inlineStr">
+        <is>
+          <t>صف 28؛ مهدي محمد القاطري؛ لوحة 7038؛ عقد HIST-XLS-T77-7038</t>
+        </is>
+      </c>
+      <c r="H15" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0048 في «عقود سابقة» على 7038 باسم ثامر محمد السيد (ساري)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="56" customHeight="1">
+      <c r="A16" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="57" t="inlineStr">
+        <is>
+          <t>رمزي الهاشمي بعزاوي</t>
+        </is>
+      </c>
+      <c r="C16" s="57" t="inlineStr">
+        <is>
+          <t>7041</t>
+        </is>
+      </c>
+      <c r="D16" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024136</t>
+        </is>
+      </c>
+      <c r="E16" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل المركبة إلى رمزي الهاشمي بعزاوي.</t>
+        </is>
+      </c>
+      <c r="F16" s="57" t="inlineStr">
+        <is>
+          <t>تحويل المركبة إلى رمزي الهاشمي بعزاوي</t>
+        </is>
+      </c>
+      <c r="G16" s="57" t="inlineStr">
+        <is>
+          <t>صف 59؛ رمزي الهاشمي بعزاوي؛ لوحة 7041؛ عقد C-ALF-0050</t>
+        </is>
+      </c>
+      <c r="H16" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024136 في «عقود سابقة» على 7041 باسم علاء الدين علي دباش — صف المعتمدون الحالي C-ALF-0050</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="56" t="inlineStr">
+        <is>
+          <t>محمد فوأد شوشان</t>
+        </is>
+      </c>
+      <c r="C17" s="56" t="inlineStr">
+        <is>
+          <t>7058</t>
+        </is>
+      </c>
+      <c r="D17" s="56" t="inlineStr">
+        <is>
+          <t>319</t>
+        </is>
+      </c>
+      <c r="E17" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="F17" s="56" t="inlineStr">
+        <is>
+          <t>تحويل إلى نشط</t>
+        </is>
+      </c>
+      <c r="G17" s="56" t="inlineStr">
+        <is>
+          <t>صف 30؛ محمد فوأد شوشان؛ لوحة 7058؛ عقد 319</t>
+        </is>
+      </c>
+      <c r="H17" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="57" t="inlineStr">
+        <is>
+          <t>مهند حمودة الظاهر</t>
+        </is>
+      </c>
+      <c r="C18" s="57" t="inlineStr">
+        <is>
+          <t>7063</t>
+        </is>
+      </c>
+      <c r="D18" s="57" t="inlineStr">
+        <is>
+          <t>AGR-055405-212</t>
+        </is>
+      </c>
+      <c r="E18" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="F18" s="57" t="inlineStr">
+        <is>
+          <t>تحويل إلى نشط</t>
+        </is>
+      </c>
+      <c r="G18" s="57" t="inlineStr">
+        <is>
+          <t>صف 31؛ مهند حمودة الظاهر؛ لوحة 7063؛ عقد AGR-055405-212</t>
+        </is>
+      </c>
+      <c r="H18" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>غير محدد في ملف المعتمدون</t>
+        </is>
+      </c>
+      <c r="C19" s="48" t="inlineStr"/>
+      <c r="D19" s="48" t="inlineStr">
+        <is>
+          <t>C-ALF-0061</t>
+        </is>
+      </c>
+      <c r="E19" s="48" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. فتح قضية. دفع دفعة واحدة 12,000.</t>
+        </is>
+      </c>
+      <c r="F19" s="48" t="inlineStr">
+        <is>
+          <t>فتح قضية + دفعة واحدة 12,000</t>
+        </is>
+      </c>
+      <c r="G19" s="48" t="inlineStr">
+        <is>
+          <t>غير موجود في المعتمدون — أُضيف هنا فقط</t>
+        </is>
+      </c>
+      <c r="H19" s="48" t="inlineStr">
+        <is>
+          <t>لا يوجد صف في المعتمدون بهذا الرقم — أُضيف في قرارات خميس فقط</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="56" customHeight="1">
+      <c r="A20" s="55" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="57" t="inlineStr">
+        <is>
+          <t>حمزة زمكيل</t>
+        </is>
+      </c>
+      <c r="C20" s="57" t="inlineStr">
+        <is>
+          <t>7071</t>
+        </is>
+      </c>
+      <c r="D20" s="57" t="inlineStr">
+        <is>
+          <t>HIST-XLS-T77-7071</t>
+        </is>
+      </c>
+      <c r="E20" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. مستعجل: كنسل المركبة + إجراء قانوني.</t>
+        </is>
+      </c>
+      <c r="F20" s="57" t="inlineStr">
+        <is>
+          <t>كنسل المركبة + إجراء قانوني (مستعجل)</t>
+        </is>
+      </c>
+      <c r="G20" s="57" t="inlineStr">
+        <is>
+          <t>صف 32؛ حمزة زمكيل؛ لوحة 7071؛ عقد HIST-XLS-T77-7071</t>
+        </is>
+      </c>
+      <c r="H20" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="55" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="56" t="inlineStr">
+        <is>
+          <t>مصطفى بالقايد</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>603353 (كانت 5892)</t>
+        </is>
+      </c>
+      <c r="D21" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0043</t>
+        </is>
+      </c>
+      <c r="E21" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. العقد صحيح. اللوحة تغيّرت إلى عادية 603353.</t>
+        </is>
+      </c>
+      <c r="F21" s="56" t="inlineStr">
+        <is>
+          <t>اعتماد العقد + تحديث اللوحة إلى 603353</t>
+        </is>
+      </c>
+      <c r="G21" s="56" t="inlineStr">
+        <is>
+          <t>صف 3؛ مصطفى بالقايد؛ لوحة 603353؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H21" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="56" customHeight="1">
+      <c r="A22" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="57" t="inlineStr">
+        <is>
+          <t>عماد العياري</t>
+        </is>
+      </c>
+      <c r="C22" s="57" t="inlineStr">
+        <is>
+          <t>11473</t>
+        </is>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024317</t>
+        </is>
+      </c>
+      <c r="E22" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل العقد إلى نشط.</t>
+        </is>
+      </c>
+      <c r="F22" s="57" t="inlineStr">
+        <is>
+          <t>تحويل إلى نشط</t>
+        </is>
+      </c>
+      <c r="G22" s="57" t="inlineStr">
+        <is>
+          <t>صف 26؛ عماد العياري؛ لوحة 11473؛ عقد LTO2024317</t>
+        </is>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="56" customHeight="1">
+      <c r="A23" s="55" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>مهدي الشريف عبد الرحيم يوسف (الاسم الحالي على LTO2024283: فهد الشريف عبد الرحيم يوسف)</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t>862165</t>
+        </is>
+      </c>
+      <c r="D23" s="56" t="inlineStr">
+        <is>
+          <t>LTO2024283</t>
+        </is>
+      </c>
+      <c r="E23" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تعديل اسم العميل إلى مهدي الشريف عبد الرحيم يوسف.</t>
+        </is>
+      </c>
+      <c r="F23" s="56" t="inlineStr">
+        <is>
+          <t>تعديل اسم العميل</t>
+        </is>
+      </c>
+      <c r="G23" s="56" t="inlineStr">
+        <is>
+          <t>صف 6؛ مهدي الشريف عبد الرحيم يوسف؛ لوحة 862165؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H23" s="56" t="inlineStr">
+        <is>
+          <t>LTO2024283 في «عقود سابقة» على 862165 باسم فهد الشريف — صف المعتمدون الحالي بلا رقم هذا العقد</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="58" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>غير محدد في ملف المعتمدون</t>
+        </is>
+      </c>
+      <c r="C24" s="48" t="inlineStr"/>
+      <c r="D24" s="48" t="inlineStr">
+        <is>
+          <t>LTO2024103</t>
+        </is>
+      </c>
+      <c r="E24" s="48" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تعديل بداية العقد إلى 1/9/2025. شطب المخالفات القديمة أو نقلها على المتسبب.</t>
+        </is>
+      </c>
+      <c r="F24" s="48" t="inlineStr">
+        <is>
+          <t>تعديل بداية العقد إلى 1/9/2025 + شطب/نقل المخالفات القديمة</t>
+        </is>
+      </c>
+      <c r="G24" s="48" t="inlineStr">
+        <is>
+          <t>غير موجود في المعتمدون — أُضيف هنا فقط</t>
+        </is>
+      </c>
+      <c r="H24" s="48" t="inlineStr">
+        <is>
+          <t>لا يوجد صف في المعتمدون بهذا الرقم — أُضيف في قرارات خميس فقط</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="56" customHeight="1">
+      <c r="A25" s="55" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="56" t="inlineStr">
+        <is>
+          <t>أمير عبد الرحمن احمد المهدى بط</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="inlineStr">
+        <is>
+          <t>847099</t>
+        </is>
+      </c>
+      <c r="D25" s="56" t="inlineStr">
+        <is>
+          <t>LTO2024124</t>
+        </is>
+      </c>
+      <c r="E25" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. فتح بلاغ + كنسل المركبة.</t>
+        </is>
+      </c>
+      <c r="F25" s="56" t="inlineStr">
+        <is>
+          <t>فتح بلاغ + كنسل المركبة</t>
+        </is>
+      </c>
+      <c r="G25" s="56" t="inlineStr">
+        <is>
+          <t>صف 33؛ أمير عبد الرحمن احمد المهدى بط؛ لوحة 847099؛ عقد LTO2024124</t>
+        </is>
+      </c>
+      <c r="H25" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="56" customHeight="1">
+      <c r="A26" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="57" t="inlineStr">
+        <is>
+          <t>الحبيب الحوسين الخليفي (صف المعتمدون على نفس اللوحة: سيف الدين محمد صالح حسين)</t>
+        </is>
+      </c>
+      <c r="C26" s="57" t="inlineStr">
+        <is>
+          <t>8204</t>
+        </is>
+      </c>
+      <c r="D26" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024150</t>
+        </is>
+      </c>
+      <c r="E26" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. فتح بلاغ مستعجل.</t>
+        </is>
+      </c>
+      <c r="F26" s="57" t="inlineStr">
+        <is>
+          <t>فتح بلاغ مستعجل</t>
+        </is>
+      </c>
+      <c r="G26" s="57" t="inlineStr">
+        <is>
+          <t>صف 16؛ سيف الدين محمد صالح حسين؛ لوحة 8204؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H26" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024150 في «عقود سابقة» على 8204 باسم الحبيب الحوسين الخليفي — ليس رقم عقد في صف المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="56" customHeight="1">
+      <c r="A27" s="55" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="56" t="inlineStr">
+        <is>
+          <t>حمد البشير يانس → حمزة البشير يانس</t>
+        </is>
+      </c>
+      <c r="C27" s="56" t="inlineStr">
+        <is>
+          <t>7043</t>
+        </is>
+      </c>
+      <c r="D27" s="56" t="inlineStr">
+        <is>
+          <t>C-ALF-0051</t>
+        </is>
+      </c>
+      <c r="E27" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تعديل الاسم في النظام: حمد البشير يانس → حمزة البشير يانس.</t>
+        </is>
+      </c>
+      <c r="F27" s="56" t="inlineStr">
+        <is>
+          <t>تعديل الاسم: حمد → حمزة البشير يانس</t>
+        </is>
+      </c>
+      <c r="G27" s="56" t="inlineStr">
+        <is>
+          <t>صف 60؛ حمد البشير يانس؛ لوحة 7043؛ عقد C-ALF-0051</t>
+        </is>
+      </c>
+      <c r="H27" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="57" t="inlineStr">
+        <is>
+          <t>بنور رقية</t>
+        </is>
+      </c>
+      <c r="C28" s="57" t="inlineStr">
+        <is>
+          <t>7060</t>
+        </is>
+      </c>
+      <c r="D28" s="57" t="inlineStr">
+        <is>
+          <t>LTO2024141</t>
+        </is>
+      </c>
+      <c r="E28" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. سيارة مفقودة.</t>
+        </is>
+      </c>
+      <c r="F28" s="57" t="inlineStr">
+        <is>
+          <t>تسجيل سيارة مفقودة</t>
+        </is>
+      </c>
+      <c r="G28" s="57" t="inlineStr">
+        <is>
+          <t>صف 64؛ بنور رقية؛ لوحة 7060؛ عقد LTO2024141</t>
+        </is>
+      </c>
+      <c r="H28" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="56" t="inlineStr">
+        <is>
+          <t>الصادق صالح إبراهيم دياب</t>
+        </is>
+      </c>
+      <c r="C29" s="56" t="inlineStr">
+        <is>
+          <t>185513</t>
+        </is>
+      </c>
+      <c r="D29" s="56" t="inlineStr">
+        <is>
+          <t>LTO20247</t>
+        </is>
+      </c>
+      <c r="E29" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. مخالفات مرورية. فتح قضية.</t>
+        </is>
+      </c>
+      <c r="F29" s="56" t="inlineStr">
+        <is>
+          <t>فتح قضية مخالفات مرورية</t>
+        </is>
+      </c>
+      <c r="G29" s="56" t="inlineStr">
+        <is>
+          <t>صف 39؛ الصادق صالح إبراهيم دياب؛ لوحة 185513؛ عقد LTO20247</t>
+        </is>
+      </c>
+      <c r="H29" s="56" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="56" customHeight="1">
+      <c r="A30" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="57" t="inlineStr">
+        <is>
+          <t>ايهاب ميرغني عوض الكريم عبد الله</t>
+        </is>
+      </c>
+      <c r="C30" s="57" t="inlineStr">
+        <is>
+          <t>185573 / 7066</t>
+        </is>
+      </c>
+      <c r="D30" s="57" t="inlineStr">
+        <is>
+          <t>C-ALF-0008</t>
+        </is>
+      </c>
+      <c r="E30" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تم دفع جميع المستحقات (حسب قرار خميس). تحويل المركبة باسمه.</t>
+        </is>
+      </c>
+      <c r="F30" s="57" t="inlineStr">
+        <is>
+          <t>تحويل المركبة باسمه (المستحقات مسددة حسب القرار)</t>
+        </is>
+      </c>
+      <c r="G30" s="57" t="inlineStr">
+        <is>
+          <t>صف 4؛ ايهاب ميرغني عوض الكريم عبد الله؛ لوحة 7066؛ عقد — | صف 40؛ ايهاب ميرغني عوض الكريم عبد الله؛ لوحة 185573؛ عقد C-ALF-0008</t>
+        </is>
+      </c>
+      <c r="H30" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56" customHeight="1">
+      <c r="A31" s="55" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="56" t="inlineStr">
+        <is>
+          <t>أسامة جريس</t>
+        </is>
+      </c>
+      <c r="C31" s="56" t="inlineStr">
+        <is>
+          <t>862169 (عقد سابق) / 846485 (صف المعتمدون)</t>
+        </is>
+      </c>
+      <c r="D31" s="56" t="inlineStr">
+        <is>
+          <t>LTO202495</t>
+        </is>
+      </c>
+      <c r="E31" s="56" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. حذف هذا العقد.</t>
+        </is>
+      </c>
+      <c r="F31" s="56" t="inlineStr">
+        <is>
+          <t>حذف العقد</t>
+        </is>
+      </c>
+      <c r="G31" s="56" t="inlineStr">
+        <is>
+          <t>صف 17؛ أسامة جريس؛ لوحة 846485؛ عقد —</t>
+        </is>
+      </c>
+      <c r="H31" s="56" t="inlineStr">
+        <is>
+          <t>LTO202495 في «عقود سابقة» على 862169 باسم أسامة جريس — صف المعتمدون الحالي لأسامة على 846485 بلا هذا الرقم</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="56" customHeight="1">
+      <c r="A32" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="57" t="inlineStr">
+        <is>
+          <t>حسن عبدالوهاب محمد الفكي</t>
+        </is>
+      </c>
+      <c r="C32" s="57" t="inlineStr">
+        <is>
+          <t>8207</t>
+        </is>
+      </c>
+      <c r="D32" s="57" t="inlineStr">
+        <is>
+          <t>C-ALF-0072</t>
+        </is>
+      </c>
+      <c r="E32" s="57" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. تحويل للشؤون القانونية. المركبة للعميل. تعديل المتأخرات فقط: 5 أشهر. سُدد 2000 من المتأخرات. المركبة بيعت → خارج الخدمة.</t>
+        </is>
+      </c>
+      <c r="F32" s="57" t="inlineStr">
+        <is>
+          <t>تحويل للشؤون + متأخرات 5 أشهر (سُدد 2000) + المركبة خارج الخدمة</t>
+        </is>
+      </c>
+      <c r="G32" s="57" t="inlineStr">
+        <is>
+          <t>صف 72؛ حسن عبدالوهاب محمد الفكي؛ لوحة 8207؛ عقد C-ALF-0072</t>
+        </is>
+      </c>
+      <c r="H32" s="57" t="inlineStr">
+        <is>
+          <t>مطابق في المعتمدون</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="59" t="inlineStr">
+        <is>
+          <t>عقود مذكورة في القرار وليست صفاً مستقلاً في المعتمدون — أُضيفت هنا حتى لا تضيع</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="56" customHeight="1">
+      <c r="A34" s="60" t="inlineStr">
+        <is>
+          <t>9ب</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>عبد العزيز بن نبيل جرفال (عقد حي على لوحة أخرى)</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>17216</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>LTO202410</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>قرار للتقرير — النظام الحي لم يُعدَّل. إلغاء LTO202410 (مرافق لقرار تحويل LTO2024340 إلى نشط).</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>إلغاء العقد</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>صف 9؛ عبد العزيز بن نبيل جرفال؛ لوحة 5890؛ عقد LTO2024340</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>ليس صفاً مستقلاً في المعتمدون — ظاهر كعقد حي على لوحة 17216 في صف 5890</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="61" t="inlineStr">
+        <is>
+          <t>دليل الألوان: أحمر رقم = لا صف في المعتمدون (أُضيف هنا فقط). برتقالي = عقد مرتبط مذكور في القرار وليس صفاً مستقلاً. عمودا «قرار خميس» و«إجراء مطلوب» أُضيفا في ورقة المعتمدون دون حذف الأعمدة القائمة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H32"/>
+  <mergeCells count="4">
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17924,7 +19750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18519,7 +20345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>